<commit_message>
Updated IND_grids_syn_5 model - 2025-10-12 14:08
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{205AF2F0-F27B-4DD8-A140-FF1DC0BF69B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F18802A-7419-45C0-9E9E-B99734A5DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11257,7 +11257,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C21868C6-ECFD-4D9B-9EF8-BD933AB4C47E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A285081-ECD2-47D4-89B4-4999EFF31566}">
   <dimension ref="B9:H358"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18255,7 +18255,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA9B8E6C-1609-4520-8A37-01585D218795}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7378E8-D018-495A-94B2-81BA053038E1}">
   <dimension ref="B9:L358"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_syn_5 model - 2025-10-12 20:49
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F18802A-7419-45C0-9E9E-B99734A5DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDE3177D-5E05-473E-8690-37FE0150A6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11257,7 +11257,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A285081-ECD2-47D4-89B4-4999EFF31566}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65475E23-F72C-4437-87C6-5FD417D138D3}">
   <dimension ref="B9:H358"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18255,7 +18255,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7378E8-D018-495A-94B2-81BA053038E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0703D0A4-6608-41C4-B372-6ED8F2A1986C}">
   <dimension ref="B9:L358"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>